<commit_message>
fix: set every Excel quotation in one font and size
Both templates now use Arial 10 throughout, keeping bold, where the export mixed Arial 8 to 14 with Calibri.
</commit_message>
<xml_diff>
--- a/config/quotation_customer_file_template.xlsx
+++ b/config/quotation_customer_file_template.xlsx
@@ -17,13 +17,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -81,15 +82,15 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>